<commit_message>
Apply updated 규칙_점수표.xlsx: 10/20/30 drop bands, 300/600 6m with sideways skip, new cuts.
</commit_message>
<xml_diff>
--- a/규칙_점수표.xlsx
+++ b/규칙_점수표.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\trade-advisor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4FBC4F4-8B55-46C3-8A8A-C4D46137720F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F4882CD-FEBB-49E5-8F83-99EF77EE4A85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="105">
   <si>
     <t>점수는 아래 항목을 하나씩 보고, 해당되면 더하거나 뺍니다.</t>
   </si>
@@ -143,12 +143,6 @@
     <t>1개월 하락률</t>
   </si>
   <si>
-    <t>한 달 동안 30% 이상 40% 미만 떨어짐</t>
-  </si>
-  <si>
-    <t>한 달 동안 40% 이상 떨어짐</t>
-  </si>
-  <si>
     <t>6개월 상승률</t>
   </si>
   <si>
@@ -194,21 +188,12 @@
     <t>제안</t>
   </si>
   <si>
-    <t>79% 이상</t>
-  </si>
-  <si>
     <t>강한 매수</t>
   </si>
   <si>
-    <t>75% 이상 ~ 79% 미만</t>
-  </si>
-  <si>
     <t>매수</t>
   </si>
   <si>
-    <t>70% 이상 ~ 75% 미만</t>
-  </si>
-  <si>
     <t>약한 매수</t>
   </si>
   <si>
@@ -218,44 +203,19 @@
     <t>홀딩</t>
   </si>
   <si>
-    <t>35% 초과 ~ 65% 미만</t>
-  </si>
-  <si>
-    <t>40% 초과 ~ 45% 이하</t>
-  </si>
-  <si>
     <t>약한 매도</t>
   </si>
   <si>
-    <t>30% 초과 ~ 35% 이하</t>
-  </si>
-  <si>
-    <t>30% 초과 ~ 40% 이하</t>
-  </si>
-  <si>
     <t>매도</t>
   </si>
   <si>
-    <t>25% 초과 ~ 30% 이하</t>
-  </si>
-  <si>
-    <t>30% 이하</t>
-  </si>
-  <si>
     <t>강한 매도</t>
   </si>
   <si>
-    <t>25% 이하</t>
-  </si>
-  <si>
     <t>6개월 동안 800% 이상 오름</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>6개월 동안 200% 이상 500% 미만 오름</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
     <t>35 이하 (너무 많이 떨어짐)</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
@@ -264,10 +224,6 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>한 달동안 10% 이상 30%미만 하락 했을 때</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
     <t>가까운 가격: 하루 변동폭의 약 55%, 또는 주가의 1.0% 중 더 작은 값.</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
@@ -356,15 +312,79 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>6개월 동안 600% 이상 오름</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
     <t>한 달 동안 70% 이상 오름</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
     <t>점수를 %로 바꾸는 법: 0점이면 0%, 15점(기본)이면 50%, 30점이면 100%.</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>67% 이상~73% 미만</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>60% 이상 ~ 67% 미만</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>73% 이상</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>33% 초과 ~ 67% 미만</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>27% 초과 ~ 33% 이하</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>20% 초과 ~ 27% 이하</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>20% 이하</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>67% 이상 ~ 73% 미만</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>73% 이상 ~ 80% 미만</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>80% 이상</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>27% 이하</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>33% 초과 ~ 37% 이하</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>6개월 동안 600% 이상 오름, 횡보 추세시 무효</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>6개월 동안 300% 이상 600% 미만 오름, 횡보 추세시 무효</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>한 달동안 10% 이상 20%미만 하락 했을 때</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>한 달 동안 20% 이상 30% 미만 떨어짐</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>한 달 동안 30% 이상 떨어짐</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -550,14 +570,14 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill>
@@ -569,13 +589,6 @@
       <fill>
         <patternFill>
           <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -885,7 +898,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="26" x14ac:dyDescent="0.65">
       <c r="A1" s="16" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="B1" s="17"/>
     </row>
@@ -917,7 +930,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.45">
@@ -1003,7 +1016,7 @@
       <c r="B2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="20">
+      <c r="C2" s="5">
         <v>15</v>
       </c>
     </row>
@@ -1014,7 +1027,7 @@
       <c r="B3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="20">
+      <c r="C3" s="5">
         <v>-1</v>
       </c>
     </row>
@@ -1034,9 +1047,9 @@
         <v>17</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="C5" s="20">
+        <v>76</v>
+      </c>
+      <c r="C5" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1067,7 +1080,7 @@
         <v>23</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="C8" s="6">
         <v>-1</v>
@@ -1075,10 +1088,10 @@
     </row>
     <row r="9" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="4" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>88</v>
+        <v>74</v>
       </c>
       <c r="C9" s="6">
         <v>1</v>
@@ -1089,7 +1102,7 @@
         <v>24</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="C10" s="6">
         <v>-1</v>
@@ -1100,7 +1113,7 @@
         <v>24</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="C11" s="6">
         <v>1</v>
@@ -1108,10 +1121,10 @@
     </row>
     <row r="12" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="4" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="C12" s="6">
         <v>1</v>
@@ -1122,9 +1135,9 @@
         <v>25</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="C13" s="20">
+        <v>79</v>
+      </c>
+      <c r="C13" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1133,7 +1146,7 @@
         <v>26</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="C14" s="6">
         <v>-2</v>
@@ -1155,9 +1168,9 @@
         <v>29</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="C16" s="20">
+        <v>81</v>
+      </c>
+      <c r="C16" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1166,9 +1179,9 @@
         <v>30</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="C17" s="20">
+        <v>82</v>
+      </c>
+      <c r="C17" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1177,7 +1190,7 @@
         <v>31</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="C18" s="6">
         <v>-1</v>
@@ -1188,9 +1201,9 @@
         <v>32</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C19" s="20">
+        <v>62</v>
+      </c>
+      <c r="C19" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1210,18 +1223,18 @@
         <v>34</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="C21" s="20">
+        <v>67</v>
+      </c>
+      <c r="C21" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="4" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="C22" s="5">
         <v>1</v>
@@ -1232,20 +1245,20 @@
         <v>35</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="C23" s="20">
+        <v>70</v>
+      </c>
+      <c r="C23" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="4" t="s">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="C24" s="20">
+        <v>85</v>
+      </c>
+      <c r="C24" s="5">
         <v>-1</v>
       </c>
     </row>
@@ -1254,7 +1267,7 @@
         <v>36</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="C25" s="6">
         <v>-1</v>
@@ -1262,10 +1275,10 @@
     </row>
     <row r="26" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="4" t="s">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>77</v>
+        <v>102</v>
       </c>
       <c r="C26" s="6">
         <v>1</v>
@@ -1276,7 +1289,7 @@
         <v>37</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>38</v>
+        <v>103</v>
       </c>
       <c r="C27" s="5">
         <v>2</v>
@@ -1287,7 +1300,7 @@
         <v>37</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>39</v>
+        <v>104</v>
       </c>
       <c r="C28" s="5">
         <v>3</v>
@@ -1295,10 +1308,10 @@
     </row>
     <row r="29" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="C29" s="6">
         <v>-3</v>
@@ -1306,7 +1319,7 @@
     </row>
     <row r="30" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>100</v>
@@ -1317,10 +1330,10 @@
     </row>
     <row r="31" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>74</v>
+        <v>101</v>
       </c>
       <c r="C31" s="6">
         <v>-1</v>
@@ -1328,10 +1341,10 @@
     </row>
     <row r="32" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C32" s="6">
         <v>-1</v>
@@ -1375,10 +1388,10 @@
     </row>
     <row r="2" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C2" s="7">
         <v>0</v>
@@ -1386,10 +1399,10 @@
     </row>
     <row r="3" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>43</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>45</v>
       </c>
       <c r="C3" s="6">
         <v>-1</v>
@@ -1397,10 +1410,10 @@
     </row>
     <row r="4" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>19</v>
@@ -1408,10 +1421,10 @@
     </row>
     <row r="5" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C5" s="7">
         <v>0</v>
@@ -1419,10 +1432,10 @@
     </row>
     <row r="6" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C6" s="6">
         <v>-1</v>
@@ -1430,10 +1443,10 @@
     </row>
     <row r="7" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C7" s="7">
         <v>0</v>
@@ -1441,7 +1454,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" s="18" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
@@ -1470,129 +1483,129 @@
   <sheetData>
     <row r="1" spans="1:5" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A1" s="19" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B1" s="17"/>
       <c r="D1" s="19" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E1" s="17"/>
     </row>
     <row r="2" spans="1:5" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="8" t="s">
-        <v>55</v>
+        <v>97</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>55</v>
+        <v>53</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>90</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="8" t="s">
-        <v>57</v>
+        <v>96</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>57</v>
+        <v>88</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="9" t="s">
-        <v>59</v>
+        <v>95</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="11" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>63</v>
+        <v>91</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="13" t="s">
-        <v>64</v>
+        <v>99</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="13" t="s">
-        <v>67</v>
+        <v>92</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="14" t="s">
-        <v>70</v>
+        <v>98</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" s="18" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
       <c r="B11" s="17"/>
       <c r="C11" s="17"/>
@@ -1601,7 +1614,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" s="18" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="B12" s="17"/>
       <c r="C12" s="17"/>

</xml_diff>

<commit_message>
Apply sheet: both-up bonus only when the 1-month uptrend line slopes down.
</commit_message>
<xml_diff>
--- a/규칙_점수표.xlsx
+++ b/규칙_점수표.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\trade-advisor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0398A3C5-4D22-43FA-A525-48EA6595CF35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83F2F238-A56A-467E-93E2-2D1EE09634DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="이렇게 봐요" sheetId="1" r:id="rId1"/>
@@ -341,10 +341,6 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>하락 추세선 상승 추세선 모두 상승이면서 해당 시점에 1개월(1시간봉기준)조회시 상승추체선이 상방향일 때, 상방향 아니면 무효</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
     <t>하방향 1개월 추세선 고려</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
@@ -354,6 +350,10 @@
   </si>
   <si>
     <t>점수를 %로 바꾸는 법: 0점이면 0%, 15점(기본)이면 50%, 31점이면 100%.</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>하락 추세선 상승 추세선 모두 상승이면서 해당 시점에 1개월(1시간봉기준)조회시 상승추체선이 하방향일 때, 상방향 아니면 무효</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -1104,10 +1104,10 @@
     </row>
     <row r="12" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>103</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="C12" s="6">
         <v>1</v>
@@ -1118,7 +1118,7 @@
         <v>101</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C13" s="6">
         <v>1</v>
@@ -1599,7 +1599,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" s="19" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B11" s="18"/>
       <c r="C11" s="18"/>

</xml_diff>

<commit_message>
Rebuild 규칙_점수표.xlsx as a clean v95 sheet matching live scoring.
</commit_message>
<xml_diff>
--- a/규칙_점수표.xlsx
+++ b/규칙_점수표.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="이렇게 봐요" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,69 +13,46 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="매수 매도 기준" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'옵션 점수'!$A$1:$C$7</definedName>
   </definedNames>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="맑은 고딕"/>
-      <charset val="129"/>
-      <family val="3"/>
       <b val="1"/>
-      <color rgb="FF1F4E79"/>
+      <color rgb="001F4E79"/>
       <sz val="18"/>
     </font>
     <font>
-      <name val="맑은 고딕"/>
-      <charset val="129"/>
-      <family val="3"/>
       <b val="1"/>
-      <color rgb="FF1F4E79"/>
+      <color rgb="001F4E79"/>
       <sz val="13"/>
     </font>
     <font>
-      <name val="맑은 고딕"/>
-      <charset val="129"/>
-      <family val="3"/>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="맑은 고딕"/>
-      <charset val="129"/>
-      <family val="3"/>
       <b val="1"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="맑은 고딕"/>
-      <charset val="129"/>
-      <family val="3"/>
       <i val="1"/>
-      <color rgb="FF666666"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="맑은 고딕"/>
-      <charset val="129"/>
-      <family val="3"/>
-      <sz val="8"/>
-      <scheme val="minor"/>
+      <color rgb="00666666"/>
     </font>
   </fonts>
   <fills count="9">
@@ -86,41 +64,41 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E79"/>
+        <fgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF8CBAD"/>
+        <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF3F4F6"/>
+        <fgColor rgb="00F3F4F6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE2EFDA"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF4B183"/>
+        <fgColor rgb="00F4B183"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -130,58 +108,25 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFE5E7EB"/>
+        <color rgb="00E5E7EB"/>
       </left>
       <right style="thin">
-        <color rgb="FFE5E7EB"/>
+        <color rgb="00E5E7EB"/>
       </right>
       <top style="thin">
-        <color rgb="FFE5E7EB"/>
+        <color rgb="00E5E7EB"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFE5E7EB"/>
+        <color rgb="00E5E7EB"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFE5E7EB"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFE5E7EB"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFE5E7EB"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FFE5E7EB"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFE5E7EB"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFE5E7EB"/>
-      </top>
-      <bottom/>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -203,6 +148,7 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -227,36 +173,10 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.3999450666829432"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.5999633777886288"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -618,119 +538,126 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="78" customWidth="1" style="18" min="1" max="1"/>
+    <col width="78" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" s="18">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>점수 규칙 (쉬운 버전) · 지금 앱 v87</t>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>점수 규칙 (쉬운 버전) · 지금 앱 v95</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n"/>
+      <c r="A2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>점수는 아래 항목을 하나씩 보고, 해당되면 더하거나 뺍니다.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>노란/초록/빨간 칸이 점수입니다. 이 칸만 고쳐서 알려주셔도 됩니다.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n"/>
-    </row>
-    <row r="6" ht="20.5" customHeight="1" s="18">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>순서</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>1. 「기본 점수」부터 「신고가 돌파 실패」까지 더합니다.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2. 더한 점수를 %로 바꿉니다. </t>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2. 더한 점수를 %로 바꿉니다. 0점이면 0%, 15점(기본)이면 50%, 31점이면 100%.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>3. %로 매수 / 매도 / 홀딩을 정합니다.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>4. 홀딩이면 끝입니다. 매수나 매도면 옵션 점수를 더하고 한 번 더 봅니다.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n"/>
-    </row>
-    <row r="12" ht="20.5" customHeight="1" s="18">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>시트 안내</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>기본 점수 — 차트·지표로 매기는 점수</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>옵션 점수 — 미국 주식만, 매수/매도일 때 추가</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>매수 매도 기준 — 몇 %면 매수이고 몇 %면 매도인지</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n"/>
-    </row>
-    <row r="17" ht="34" customHeight="1" s="18">
-      <c r="A17" s="1" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>참고: 6개월 상승률은 180일 전 종가 대비입니다. 그날이 주말·휴장이면 근처 거래일 종가를 씁니다.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="34" customHeight="1" s="18">
-      <c r="A18" s="1" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>3개월 이상 조회에서 1개월 창(상승선·1개월 추세)은 일봉이 아니라 1개월 조회와 같은 1시간봉 30일을 씁니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>1개월 조회 상승선은 마지막 스윙 저점 두 개, 6개월(3개월·1년) 상승선은 중간 저점이 안 깨는 상승 지지선입니다.</t>
         </is>
       </c>
     </row>
@@ -749,550 +676,578 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C35"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25.6640625" customWidth="1" style="18" min="1" max="1"/>
-    <col width="107.58203125" customWidth="1" style="18" min="2" max="2"/>
-    <col width="10" customWidth="1" style="18" min="3" max="3"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" s="18">
-      <c r="A1" s="20" t="inlineStr">
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="B1" s="20" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>이럴 때</t>
         </is>
       </c>
-      <c r="C1" s="20" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>점수</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="32" customHeight="1" s="18">
-      <c r="A2" s="4" t="inlineStr">
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>기본</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>시작할 때 항상 줌</t>
         </is>
       </c>
-      <c r="C2" s="5" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" ht="32" customHeight="1" s="18">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>+15</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>추세</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>조회 기간이 1~2개월이고, 상승 추세</t>
         </is>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="7" t="n">
         <v>-1</v>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1" s="18">
-      <c r="A4" s="4" t="inlineStr">
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>추세</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>조회 기간이 1~2개월이고, 하락 추세</t>
         </is>
       </c>
-      <c r="C4" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" ht="32" customHeight="1" s="18">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>추세</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>조회 기간이 3개월 이상이고, 하락 추세 (눌림)</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" ht="32" customHeight="1" s="18">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>추세</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>조회 기간이 3개월 이상이고, 상승 추세 (고점 추격)</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="7" t="n">
         <v>-1</v>
       </c>
     </row>
-    <row r="7" ht="32" customHeight="1" s="18">
-      <c r="A7" s="4" t="inlineStr">
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>추세</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>횡보일 때</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="8" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="8" ht="32" customHeight="1" s="18">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>하락 추세선 근접</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>하락 추세선에 근접 했을 때, 돌파하면 무효</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="7" t="n">
         <v>-1</v>
       </c>
     </row>
-    <row r="9" ht="32" customHeight="1" s="18">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>상승 추세선 근접</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>상승 추세선 근접 했을 때, 이탈하면 무효</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" ht="32" customHeight="1" s="18">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>추세선 방향</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>하락 추세선 상승 추세선 모두 하락이면서 현재가가 하락 추세선 근접했을때, 하락 추세선 돌파시 무효</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n">
+      <c r="C10" s="7" t="n">
         <v>-1</v>
       </c>
     </row>
-    <row r="11" ht="32" customHeight="1" s="18">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>추세선 방향</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>하락 추세선 상승 추세선 모두 하락이면서 현재가가 상승 추세선 근접했을 때, 상승 추세선 이탈시 무효</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" ht="32" customHeight="1" s="18">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>하방향 1개월 추세선 고려</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>(3개월,6개월,1년 조회에만 적용) 하락 추세선 상승 추세선 모두 하락이면서 해당 시점에 1개월(1시간봉기준)조회시 상승추체선이 상방향일 때, 상방향 아니면 무효</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1" s="18">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>(3개월,6개월,1년 조회에만 적용) 하락 추세선 상승 추세선 모두 하락이면서 해당 시점에 1개월(1시간봉기준)조회시 상승추세선이 상방향일 때, 상방향 아니면 무효</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>상방향 1개월 추세선 고려</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>(3개월,6개월,1년 조회에만 적용) 하락 추세선 상승 추세선 모두 상승이면서 해당 시점에 1개월(1시간봉기준)조회시 상승추체선이 하방향일 때, 상방향 아니면 무효</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" ht="32" customHeight="1" s="18">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>(3개월,6개월,1년 조회에만 적용) 하락 추세선 상승 추세선 모두 상승이면서 해당 시점에 1개월(1시간봉기준)조회시 상승추세선이 하방향일 때, 하방향 아니면 무효</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>지지 근접</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>지지선 바로 옆이고 강도 4 이상일 때</t>
         </is>
       </c>
-      <c r="C14" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" ht="32" customHeight="1" s="18">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>지지 이탈</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>지지 이탈 후 다음 지지선이 현재가 보다 뚜렷이 아래에 있을 때</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n">
+      <c r="C15" s="7" t="n">
         <v>-2</v>
       </c>
     </row>
-    <row r="16" ht="32" customHeight="1" s="18">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>저항 근접</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>저항선 바로 옆이고, 강도 4 이상일 때</t>
         </is>
       </c>
-      <c r="C16" s="6" t="n">
+      <c r="C16" s="7" t="n">
         <v>-1</v>
       </c>
     </row>
-    <row r="17" ht="32" customHeight="1" s="18">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>최대 매물 (POC)</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>현재가가 거래가 가장 많았던 가격 근접 했을 때, 이탈 시 무효</t>
         </is>
       </c>
-      <c r="C17" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" ht="32" customHeight="1" s="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>밸류 하단 (VAL)</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>현재가가 싼 구간 아래이고, 상승 추세일 때</t>
         </is>
       </c>
-      <c r="C18" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" ht="32" customHeight="1" s="18">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>밸류 상단 (VAH)</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>현재가가 비싼 구간 위, 돌파시 무효</t>
         </is>
       </c>
-      <c r="C19" s="6" t="n">
+      <c r="C19" s="7" t="n">
         <v>-1</v>
       </c>
     </row>
-    <row r="20" ht="32" customHeight="1" s="18">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>RSI</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>35 이하 (너무 많이 떨어짐)</t>
         </is>
       </c>
-      <c r="C20" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" ht="32" customHeight="1" s="18">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>RSI</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>70 이상 (너무 많이 오름)</t>
         </is>
       </c>
-      <c r="C21" s="6" t="n">
+      <c r="C21" s="7" t="n">
         <v>-1</v>
       </c>
     </row>
-    <row r="22" ht="32" customHeight="1" s="18">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>20일선</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>현재가가 20일선 근처일때, 20일선 완전 이탈시 무효</t>
         </is>
       </c>
-      <c r="C22" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" ht="32" customHeight="1" s="18">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>60일선</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>현재가가 60일선 근처일때, 60일선 완전 이탈시 무효</t>
         </is>
       </c>
-      <c r="C23" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" ht="32" customHeight="1" s="18">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="32" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>180일선</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>현재가가 장기 이평 근처일 때. 6개월 조회는 180일선, 1년 조회는 300일선, 완전이탈시 무효</t>
         </is>
       </c>
-      <c r="C24" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" ht="32" customHeight="1" s="18">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="32" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>20일선 60일선 교차</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>20일선 방향이 하방으로 떨어지면서 60일선 아래로 떨어지기 시작할때, 떨어지고 4봉이상 지나면 무효</t>
         </is>
       </c>
-      <c r="C25" s="5" t="n">
+      <c r="C25" s="7" t="n">
         <v>-1</v>
       </c>
     </row>
-    <row r="26" ht="32" customHeight="1" s="18">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>1개월 상승률</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>한 달 동안 70% 이상 오름</t>
         </is>
       </c>
-      <c r="C26" s="6" t="n">
+      <c r="C26" s="7" t="n">
         <v>-1</v>
       </c>
     </row>
-    <row r="27" ht="32" customHeight="1" s="18">
-      <c r="A27" s="4" t="inlineStr">
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>1개월 하락률</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>한 달동안 10% 이상 20%미만 하락 했을 때</t>
         </is>
       </c>
-      <c r="C27" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" ht="32" customHeight="1" s="18">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>1개월 하락률</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>한 달 동안 20% 이상 30% 미만 떨어짐</t>
         </is>
       </c>
-      <c r="C28" s="5" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="29" ht="32" customHeight="1" s="18">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>+2</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="32" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>1개월 하락률</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>한 달 동안 30% 이상 떨어짐</t>
         </is>
       </c>
-      <c r="C29" s="5" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="30" ht="32" customHeight="1" s="18">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>+3</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="32" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>6개월 상승률</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>6개월 동안 800% 이상 오름</t>
         </is>
       </c>
-      <c r="C30" s="6" t="n">
+      <c r="C30" s="7" t="n">
         <v>-3</v>
       </c>
     </row>
-    <row r="31" ht="32" customHeight="1" s="18">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="31" ht="32" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>6개월 상승률</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>6개월 동안 600% 이상 오름, 횡보 추세나 하락 추세시 무효</t>
         </is>
       </c>
-      <c r="C31" s="6" t="n">
+      <c r="C31" s="7" t="n">
         <v>-2</v>
       </c>
     </row>
-    <row r="32" ht="32" customHeight="1" s="18">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="32" ht="32" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>6개월 상승률</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>6개월 동안 300% 이상 600% 미만 오름, 횡보 추세나 하락 추세시 무효</t>
         </is>
       </c>
-      <c r="C32" s="6" t="n">
+      <c r="C32" s="7" t="n">
         <v>-1</v>
       </c>
     </row>
-    <row r="33" ht="32" customHeight="1" s="18">
-      <c r="A33" s="4" t="inlineStr">
+    <row r="33" ht="32" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>단기 급상승</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>1개 봉만에 20% 이상 상승했을 시</t>
         </is>
       </c>
-      <c r="C33" s="6" t="n">
+      <c r="C33" s="7" t="n">
         <v>-1</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="34" ht="32" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>신고가</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>위에 저항이 아예 없는 신고가의 경우 +1점, 신고가 이후 4개봉 지나면 무효</t>
         </is>
       </c>
-      <c r="C34" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="32" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>신고가 돌파 실패</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>신고가 이후 8개봉동안 신고가 갱신 못하면 -1점, 신고가 이후 12개봉 지나면 무효</t>
         </is>
       </c>
-      <c r="C35" s="6" t="n">
+      <c r="C35" s="7" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C33"/>
-  <conditionalFormatting sqref="C2:C1048576">
-    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
+  <autoFilter ref="A1:C35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1304,124 +1259,124 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" style="18" min="1" max="1"/>
-    <col width="78" customWidth="1" style="18" min="2" max="2"/>
-    <col width="10" customWidth="1" style="18" min="3" max="3"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" s="18">
-      <c r="A1" s="20" t="inlineStr">
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="B1" s="20" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>이럴 때</t>
         </is>
       </c>
-      <c r="C1" s="20" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>점수</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="32" customHeight="1" s="18">
-      <c r="A2" s="4" t="inlineStr">
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>옵션</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>기존 결과가 홀딩이면 옵션은 보지 않음</t>
         </is>
       </c>
-      <c r="C2" s="7" t="n">
+      <c r="C2" s="8" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="3" ht="32" customHeight="1" s="18">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>옵션</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>기존이 매도인데, 만기가 14일 안이고, 위쪽에 콜 벽이 두껍고 아래 풋 벽이 얇음</t>
         </is>
       </c>
-      <c r="C3" s="6" t="n">
+      <c r="C3" s="7" t="n">
         <v>-1</v>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1" s="18">
-      <c r="A4" s="4" t="inlineStr">
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>옵션</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>기존이 매도인데, 반대로 아래 풋 벽이 두껍고 위 콜 벽이 얇음</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>+1</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1" s="18">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>옵션</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>기존이 매도인데, 벽이 멀거나 둘 다 얇음</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="8" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1" s="18">
-      <c r="A6" s="4" t="inlineStr">
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>옵션</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>기존이 매수인데, 아래 풋 벽이 얇고 위 콜 벽이 두꺼움</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="7" t="n">
         <v>-1</v>
       </c>
     </row>
-    <row r="7" ht="32" customHeight="1" s="18">
-      <c r="A7" s="4" t="inlineStr">
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>옵션</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>기존이 매수인데, 위와 다르면</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="8" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>참고: 미국 주식, 오늘 조회만. 근처는 현재가에서 5% 안, 멀면 8% 밖.</t>
         </is>
@@ -1443,214 +1398,212 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" style="18" min="1" max="1"/>
-    <col width="14" customWidth="1" style="18" min="2" max="2"/>
-    <col width="4" customWidth="1" style="18" min="3" max="3"/>
-    <col width="28" customWidth="1" style="18" min="4" max="4"/>
-    <col width="14" customWidth="1" style="18" min="5" max="5"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.5" customHeight="1" s="18">
-      <c r="A1" s="20" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>코인</t>
         </is>
       </c>
-      <c r="B1" s="21" t="n"/>
-      <c r="D1" s="20" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>주식</t>
         </is>
       </c>
-      <c r="E1" s="21" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1" s="18">
-      <c r="A2" s="20" t="inlineStr">
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>합산 %</t>
         </is>
       </c>
-      <c r="B2" s="20" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>제안</t>
         </is>
       </c>
-      <c r="D2" s="20" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>합산 %</t>
         </is>
       </c>
-      <c r="E2" s="20" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>제안</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="28" customHeight="1" s="18">
-      <c r="A3" s="8" t="inlineStr">
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>80% 이상</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>강한 매수</t>
         </is>
       </c>
-      <c r="D3" s="16" t="inlineStr">
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>73% 이상</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>강한 매수</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="28" customHeight="1" s="18">
-      <c r="A4" s="8" t="inlineStr">
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>73% 이상 ~ 80% 미만</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>매수</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>67% 이상~73% 미만</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>67% 이상 ~ 73% 미만</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>매수</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1" s="18">
-      <c r="A5" s="9" t="inlineStr">
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>67% 이상 ~ 73% 미만</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>약한 매수</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="11" t="inlineStr">
         <is>
           <t>60% 이상 ~ 67% 미만</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>약한 매수</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="28" customHeight="1" s="18">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>45% 초과 ~ 70% 미만</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>37% 초과 ~ 67% 미만</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>홀딩</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
-        <is>
-          <t>33% 초과 ~ 67% 미만</t>
-        </is>
-      </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>33% 초과 ~ 60% 미만</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>홀딩</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1" s="18">
-      <c r="A7" s="13" t="inlineStr">
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>33% 초과 ~ 37% 이하</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>약한 매도</t>
         </is>
       </c>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>27% 초과 ~ 33% 이하</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>약한 매도</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1" s="18">
-      <c r="A8" s="13" t="inlineStr">
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>27% 초과 ~ 33% 이하</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>매도</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="D8" s="15" t="inlineStr">
         <is>
           <t>20% 초과 ~ 27% 이하</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>매도</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1" s="18">
-      <c r="A9" s="14" t="inlineStr">
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>27% 이하</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>강한 매도</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="D9" s="16" t="inlineStr">
         <is>
           <t>20% 이하</t>
         </is>
       </c>
-      <c r="E9" s="15" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>강한 매도</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>점수를 %로 바꾸는 법: 0점이면 0%, 15점(기본)이면 50%, 31점이면 100%.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>가까운 가격: 하루 변동폭의 약 55%, 또는 주가의 1.0% 중 더 큰 값.</t>
         </is>

</xml_diff>

<commit_message>
Apply sheet v97: ATH hit/resist/reenter and 1-month bonus only when near the uptrend line.
</commit_message>
<xml_diff>
--- a/규칙_점수표.xlsx
+++ b/규칙_점수표.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\trade-advisor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABD0DB4C-99BD-4C7A-9DFB-C377D5135B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EB46768-B4B4-41EF-8BBD-A163E1149160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19040" yWindow="800" windowWidth="18110" windowHeight="19320" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="이렇게 봐요" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="106">
   <si>
     <t>점수는 아래 항목을 하나씩 보고, 해당되면 더하거나 뺍니다.</t>
   </si>
@@ -113,15 +113,9 @@
     <t>하방향 1개월 추세선 고려</t>
   </si>
   <si>
-    <t>(3개월,6개월,1년 조회에만 적용) 하락 추세선 상승 추세선 모두 하락이면서 해당 시점에 1개월(1시간봉기준)조회시 상승추세선이 상방향일 때, 상방향 아니면 무효</t>
-  </si>
-  <si>
     <t>상방향 1개월 추세선 고려</t>
   </si>
   <si>
-    <t>(3개월,6개월,1년 조회에만 적용) 하락 추세선 상승 추세선 모두 상승이면서 해당 시점에 1개월(1시간봉기준)조회시 상승추세선이 하방향일 때, 하방향 아니면 무효</t>
-  </si>
-  <si>
     <t>지지 근접</t>
   </si>
   <si>
@@ -227,18 +221,6 @@
     <t>1개 봉만에 20% 이상 상승했을 시</t>
   </si>
   <si>
-    <t>신고가</t>
-  </si>
-  <si>
-    <t>위에 저항이 아예 없는 신고가의 경우 +1점, 신고가 이후 4개봉 지나면 무효</t>
-  </si>
-  <si>
-    <t>신고가 돌파 실패</t>
-  </si>
-  <si>
-    <t>신고가 이후 8개봉동안 신고가 갱신 못하면 -1점, 신고가 이후 12개봉 지나면 무효</t>
-  </si>
-  <si>
     <t>옵션</t>
   </si>
   <si>
@@ -332,15 +314,47 @@
     <t>가까운 가격: 하루 변동폭의 약 55%, 또는 주가의 1.0% 중 더 큰 값.</t>
   </si>
   <si>
-    <t>점수를 %로 바꾸는 법: 1점이면 0%, 15점(기본)이면 50%, 30점이면 100%.</t>
+    <t>33% 초과 ~ 60% 미만</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>점수 규칙 (쉬운 버전) · 지금 앱 v96</t>
+    <t>(3개월,6개월,1년 조회에만 적용) 하락 추세선 상승 추세선 모두 하락이면서 해당 시점에 1개월(1시간봉기준)조회시 상승추세선이 상방향일 때</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>33% 초과 ~ 60% 미만</t>
+    <t>(3개월,6개월,1년 조회에만 적용) 하락 추세선 상승 추세선 모두 상승이면서 해당 시점에 1개월(1시간봉기준)조회시 상승추세선이 하방향일 때 상승 추세선에 근접했으면 가점, 하방향 아니면 무효</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>점수 규칙 (쉬운 버전) · 지금 앱 v97</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>신고가 저항</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>신고가 달성</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>6개월 상승률이 800% 이상이면서 위에 저항이 없는 신고가의 경우</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>6개월 상승률이 800% 미만이면서 위에 저항이 없는 신고가의 경우</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>신고가 이탈</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>신고가 돌파 후 다시 하락 추세선 안으로 현재가가 내려왔을 때</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>점수를 %로 바꾸는 법: 0점이면 0%, 15점(기본)이면 50%, 30점이면 100%.</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -473,7 +487,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -524,9 +538,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -839,7 +850,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="26" x14ac:dyDescent="0.65">
       <c r="A1" s="16" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B1" s="17"/>
     </row>
@@ -936,7 +947,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -962,7 +973,7 @@
       <c r="B2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="20">
+      <c r="C2" s="5">
         <v>15</v>
       </c>
     </row>
@@ -984,7 +995,7 @@
       <c r="B4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="20">
+      <c r="C4" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1006,7 +1017,7 @@
       <c r="B6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="20">
+      <c r="C6" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1015,40 +1026,40 @@
         <v>27</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" s="20">
+        <v>96</v>
+      </c>
+      <c r="C7" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" s="20">
+        <v>97</v>
+      </c>
+      <c r="C8" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" s="20">
+        <v>30</v>
+      </c>
+      <c r="C9" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C10" s="6">
         <v>-2</v>
@@ -1056,10 +1067,10 @@
     </row>
     <row r="11" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C11" s="6">
         <v>-1</v>
@@ -1067,32 +1078,32 @@
     </row>
     <row r="12" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C12" s="20">
+        <v>36</v>
+      </c>
+      <c r="C12" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" s="20">
+        <v>38</v>
+      </c>
+      <c r="C13" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C14" s="6">
         <v>-1</v>
@@ -1100,21 +1111,21 @@
     </row>
     <row r="15" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C15" s="20">
+        <v>42</v>
+      </c>
+      <c r="C15" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>43</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>45</v>
       </c>
       <c r="C16" s="6">
         <v>-1</v>
@@ -1122,43 +1133,43 @@
     </row>
     <row r="17" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C17" s="20">
+        <v>45</v>
+      </c>
+      <c r="C17" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C18" s="20">
+        <v>47</v>
+      </c>
+      <c r="C18" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C19" s="20">
+        <v>49</v>
+      </c>
+      <c r="C19" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C20" s="6">
         <v>-1</v>
@@ -1166,10 +1177,10 @@
     </row>
     <row r="21" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C21" s="6">
         <v>-1</v>
@@ -1177,43 +1188,43 @@
     </row>
     <row r="22" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C22" s="20">
+        <v>55</v>
+      </c>
+      <c r="C22" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B23" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B23" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C23" s="20">
+      <c r="C23" s="5">
         <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C24" s="20">
+        <v>57</v>
+      </c>
+      <c r="C24" s="5">
         <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C25" s="6">
         <v>-3</v>
@@ -1221,10 +1232,10 @@
     </row>
     <row r="26" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B26" s="4" t="s">
         <v>60</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>62</v>
       </c>
       <c r="C26" s="6">
         <v>-2</v>
@@ -1232,10 +1243,10 @@
     </row>
     <row r="27" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C27" s="6">
         <v>-1</v>
@@ -1243,10 +1254,10 @@
     </row>
     <row r="28" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="4" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C28" s="6">
         <v>-1</v>
@@ -1254,23 +1265,34 @@
     </row>
     <row r="29" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="4" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="C29" s="20">
+        <v>102</v>
+      </c>
+      <c r="C29" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="4" t="s">
-        <v>68</v>
+        <v>99</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>69</v>
+        <v>101</v>
       </c>
       <c r="C30" s="6">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A31" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C31" s="6">
         <v>-1</v>
       </c>
     </row>
@@ -1304,10 +1326,10 @@
     </row>
     <row r="2" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="4" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="C2" s="7">
         <v>0</v>
@@ -1315,10 +1337,10 @@
     </row>
     <row r="3" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="4" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="C3" s="6">
         <v>-1</v>
@@ -1326,10 +1348,10 @@
     </row>
     <row r="4" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="4" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>19</v>
@@ -1337,10 +1359,10 @@
     </row>
     <row r="5" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="4" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C5" s="7">
         <v>0</v>
@@ -1348,10 +1370,10 @@
     </row>
     <row r="6" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C6" s="6">
         <v>-1</v>
@@ -1359,10 +1381,10 @@
     </row>
     <row r="7" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>70</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>76</v>
       </c>
       <c r="C7" s="7">
         <v>0</v>
@@ -1370,7 +1392,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" s="18" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
@@ -1399,129 +1421,129 @@
   <sheetData>
     <row r="1" spans="1:5" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A1" s="19" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="B1" s="17"/>
       <c r="D1" s="19" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="E1" s="17"/>
     </row>
     <row r="2" spans="1:5" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="8" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="8" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="9" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="11" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="13" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="13" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="14" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" s="18" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B11" s="17"/>
       <c r="C11" s="17"/>
@@ -1530,7 +1552,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" s="18" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="B12" s="17"/>
       <c r="C12" s="17"/>

</xml_diff>

<commit_message>
Apply sheet v98: 15/25/35 one-month drop bands and ATR 30% near distance.
</commit_message>
<xml_diff>
--- a/규칙_점수표.xlsx
+++ b/규칙_점수표.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\trade-advisor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EB46768-B4B4-41EF-8BBD-A163E1149160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{114804E5-9017-4F9F-AF9F-BC89375AEED0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19040" yWindow="800" windowWidth="18110" windowHeight="19320" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19040" yWindow="800" windowWidth="18110" windowHeight="19320" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="이렇게 봐요" sheetId="1" r:id="rId1"/>
@@ -194,15 +194,6 @@
     <t>1개월 하락률</t>
   </si>
   <si>
-    <t>한 달동안 10% 이상 20%미만 하락 했을 때</t>
-  </si>
-  <si>
-    <t>한 달 동안 20% 이상 30% 미만 떨어짐</t>
-  </si>
-  <si>
-    <t>한 달 동안 30% 이상 떨어짐</t>
-  </si>
-  <si>
     <t>6개월 상승률</t>
   </si>
   <si>
@@ -309,9 +300,6 @@
   </si>
   <si>
     <t>20% 이하</t>
-  </si>
-  <si>
-    <t>가까운 가격: 하루 변동폭의 약 55%, 또는 주가의 1.0% 중 더 큰 값.</t>
   </si>
   <si>
     <t>33% 초과 ~ 60% 미만</t>
@@ -326,10 +314,6 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>점수 규칙 (쉬운 버전) · 지금 앱 v97</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
     <t>신고가 저항</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
@@ -355,6 +339,26 @@
   </si>
   <si>
     <t>점수를 %로 바꾸는 법: 0점이면 0%, 15점(기본)이면 50%, 30점이면 100%.</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>가까운 가격: 하루 변동폭의 약 30%, 또는 주가의 1.0% 중 더 큰 값.</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>한 달동안 15% 이상 25%미만 하락 했을 때</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>한 달 동안 25% 이상 35% 미만 떨어짐</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>한 달 동안 35% 이상 떨어짐</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>점수 규칙 (쉬운 버전) · 지금 앱 v98</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -850,7 +854,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="26" x14ac:dyDescent="0.65">
       <c r="A1" s="16" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="B1" s="17"/>
     </row>
@@ -1026,7 +1030,7 @@
         <v>27</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C7" s="5">
         <v>1</v>
@@ -1037,7 +1041,7 @@
         <v>28</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C8" s="5">
         <v>1</v>
@@ -1191,7 +1195,7 @@
         <v>54</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>55</v>
+        <v>102</v>
       </c>
       <c r="C22" s="5">
         <v>1</v>
@@ -1202,7 +1206,7 @@
         <v>54</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>56</v>
+        <v>103</v>
       </c>
       <c r="C23" s="5">
         <v>2</v>
@@ -1213,7 +1217,7 @@
         <v>54</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>57</v>
+        <v>104</v>
       </c>
       <c r="C24" s="5">
         <v>3</v>
@@ -1221,10 +1225,10 @@
     </row>
     <row r="25" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C25" s="6">
         <v>-3</v>
@@ -1232,10 +1236,10 @@
     </row>
     <row r="26" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C26" s="6">
         <v>-2</v>
@@ -1243,10 +1247,10 @@
     </row>
     <row r="27" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" s="4" t="s">
         <v>58</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>61</v>
       </c>
       <c r="C27" s="6">
         <v>-1</v>
@@ -1254,10 +1258,10 @@
     </row>
     <row r="28" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C28" s="6">
         <v>-1</v>
@@ -1265,10 +1269,10 @@
     </row>
     <row r="29" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="4" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C29" s="5">
         <v>1</v>
@@ -1276,10 +1280,10 @@
     </row>
     <row r="30" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="4" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="C30" s="6">
         <v>-1</v>
@@ -1287,10 +1291,10 @@
     </row>
     <row r="31" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="4" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="C31" s="6">
         <v>-1</v>
@@ -1326,10 +1330,10 @@
     </row>
     <row r="2" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C2" s="7">
         <v>0</v>
@@ -1337,10 +1341,10 @@
     </row>
     <row r="3" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C3" s="6">
         <v>-1</v>
@@ -1348,10 +1352,10 @@
     </row>
     <row r="4" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>64</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>67</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>19</v>
@@ -1359,10 +1363,10 @@
     </row>
     <row r="5" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C5" s="7">
         <v>0</v>
@@ -1370,10 +1374,10 @@
     </row>
     <row r="6" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C6" s="6">
         <v>-1</v>
@@ -1381,10 +1385,10 @@
     </row>
     <row r="7" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C7" s="7">
         <v>0</v>
@@ -1392,7 +1396,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" s="18" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
@@ -1421,129 +1425,129 @@
   <sheetData>
     <row r="1" spans="1:5" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A1" s="19" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B1" s="17"/>
       <c r="D1" s="19" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E1" s="17"/>
     </row>
     <row r="2" spans="1:5" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="8" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="8" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="9" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="11" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="13" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="13" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="14" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" s="18" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="B11" s="17"/>
       <c r="C11" s="17"/>
@@ -1552,7 +1556,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" s="18" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="B12" s="17"/>
       <c r="C12" s="17"/>

</xml_diff>

<commit_message>
Apply sheet v99: drop 1-month rally penalty, skip 800% off uptrend, and time-limit ATH items.
</commit_message>
<xml_diff>
--- a/규칙_점수표.xlsx
+++ b/규칙_점수표.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\trade-advisor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{114804E5-9017-4F9F-AF9F-BC89375AEED0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D509FC9D-7DD2-4226-87A1-A21F8E72413F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19040" yWindow="800" windowWidth="18110" windowHeight="19320" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="이렇게 봐요" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="매수 매도 기준" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'옵션 점수'!$A$1:$C$7</definedName>
   </definedNames>
   <calcPr calcId="0"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="104">
   <si>
     <t>점수는 아래 항목을 하나씩 보고, 해당되면 더하거나 뺍니다.</t>
   </si>
@@ -38,9 +38,6 @@
     <t>순서</t>
   </si>
   <si>
-    <t>1. 「기본 점수」부터 「신고가 돌파 실패」까지 더합니다.</t>
-  </si>
-  <si>
     <t>2. 더한 점수를 %로 바꿉니다. 0점이면 0%, 15점(기본)이면 50%, 31점이면 100%.</t>
   </si>
   <si>
@@ -185,180 +182,181 @@
     <t>20일선 방향이 하방으로 떨어지면서 60일선 아래로 떨어지기 시작할때, 떨어지고 4봉이상 지나면 무효</t>
   </si>
   <si>
-    <t>1개월 상승률</t>
-  </si>
-  <si>
-    <t>한 달 동안 70% 이상 오름</t>
-  </si>
-  <si>
     <t>1개월 하락률</t>
   </si>
   <si>
     <t>6개월 상승률</t>
   </si>
   <si>
-    <t>6개월 동안 800% 이상 오름</t>
-  </si>
-  <si>
     <t>6개월 동안 600% 이상 오름, 횡보 추세나 하락 추세시 무효</t>
   </si>
   <si>
+    <t>단기 급상승</t>
+  </si>
+  <si>
+    <t>옵션</t>
+  </si>
+  <si>
+    <t>기존 결과가 홀딩이면 옵션은 보지 않음</t>
+  </si>
+  <si>
+    <t>기존이 매도인데, 만기가 14일 안이고, 위쪽에 콜 벽이 두껍고 아래 풋 벽이 얇음</t>
+  </si>
+  <si>
+    <t>기존이 매도인데, 반대로 아래 풋 벽이 두껍고 위 콜 벽이 얇음</t>
+  </si>
+  <si>
+    <t>기존이 매도인데, 벽이 멀거나 둘 다 얇음</t>
+  </si>
+  <si>
+    <t>기존이 매수인데, 아래 풋 벽이 얇고 위 콜 벽이 두꺼움</t>
+  </si>
+  <si>
+    <t>기존이 매수인데, 위와 다르면</t>
+  </si>
+  <si>
+    <t>참고: 미국 주식, 오늘 조회만. 근처는 현재가에서 5% 안, 멀면 8% 밖.</t>
+  </si>
+  <si>
+    <t>코인</t>
+  </si>
+  <si>
+    <t>주식</t>
+  </si>
+  <si>
+    <t>합산 %</t>
+  </si>
+  <si>
+    <t>제안</t>
+  </si>
+  <si>
+    <t>80% 이상</t>
+  </si>
+  <si>
+    <t>강한 매수</t>
+  </si>
+  <si>
+    <t>73% 이상</t>
+  </si>
+  <si>
+    <t>73% 이상 ~ 80% 미만</t>
+  </si>
+  <si>
+    <t>매수</t>
+  </si>
+  <si>
+    <t>67% 이상 ~ 73% 미만</t>
+  </si>
+  <si>
+    <t>약한 매수</t>
+  </si>
+  <si>
+    <t>60% 이상 ~ 67% 미만</t>
+  </si>
+  <si>
+    <t>37% 초과 ~ 67% 미만</t>
+  </si>
+  <si>
+    <t>홀딩</t>
+  </si>
+  <si>
+    <t>33% 초과 ~ 37% 이하</t>
+  </si>
+  <si>
+    <t>약한 매도</t>
+  </si>
+  <si>
+    <t>27% 초과 ~ 33% 이하</t>
+  </si>
+  <si>
+    <t>매도</t>
+  </si>
+  <si>
+    <t>20% 초과 ~ 27% 이하</t>
+  </si>
+  <si>
+    <t>27% 이하</t>
+  </si>
+  <si>
+    <t>강한 매도</t>
+  </si>
+  <si>
+    <t>20% 이하</t>
+  </si>
+  <si>
+    <t>33% 초과 ~ 60% 미만</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>(3개월,6개월,1년 조회에만 적용) 하락 추세선 상승 추세선 모두 하락이면서 해당 시점에 1개월(1시간봉기준)조회시 상승추세선이 상방향일 때</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>(3개월,6개월,1년 조회에만 적용) 하락 추세선 상승 추세선 모두 상승이면서 해당 시점에 1개월(1시간봉기준)조회시 상승추세선이 하방향일 때 상승 추세선에 근접했으면 가점, 하방향 아니면 무효</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>신고가 저항</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>신고가 달성</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>신고가 이탈</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>가까운 가격: 하루 변동폭의 약 30%, 또는 주가의 1.0% 중 더 큰 값.</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>한 달동안 15% 이상 25%미만 하락 했을 때</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>한 달 동안 25% 이상 35% 미만 떨어짐</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>한 달 동안 35% 이상 떨어짐</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>6개월 상승률이 800% 미만이면서 위에 저항이 없는 신고가의 경우, 3봉 이후 무효</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>6개월 상승률이 800% 이상이면서 위에 저항이 없는 신고가의 경우, 2봉 이후 무효</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>신고가 돌파 후 3봉 이내에 다시 하락 추세선 안으로 현재가가 내려왔을 때, 3봉 이후 무효</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>1개 봉만에 20% 이상 상승했을 시</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
     <t>6개월 동안 300% 이상 600% 미만 오름, 횡보 추세나 하락 추세시 무효</t>
-  </si>
-  <si>
-    <t>단기 급상승</t>
-  </si>
-  <si>
-    <t>1개 봉만에 20% 이상 상승했을 시</t>
-  </si>
-  <si>
-    <t>옵션</t>
-  </si>
-  <si>
-    <t>기존 결과가 홀딩이면 옵션은 보지 않음</t>
-  </si>
-  <si>
-    <t>기존이 매도인데, 만기가 14일 안이고, 위쪽에 콜 벽이 두껍고 아래 풋 벽이 얇음</t>
-  </si>
-  <si>
-    <t>기존이 매도인데, 반대로 아래 풋 벽이 두껍고 위 콜 벽이 얇음</t>
-  </si>
-  <si>
-    <t>기존이 매도인데, 벽이 멀거나 둘 다 얇음</t>
-  </si>
-  <si>
-    <t>기존이 매수인데, 아래 풋 벽이 얇고 위 콜 벽이 두꺼움</t>
-  </si>
-  <si>
-    <t>기존이 매수인데, 위와 다르면</t>
-  </si>
-  <si>
-    <t>참고: 미국 주식, 오늘 조회만. 근처는 현재가에서 5% 안, 멀면 8% 밖.</t>
-  </si>
-  <si>
-    <t>코인</t>
-  </si>
-  <si>
-    <t>주식</t>
-  </si>
-  <si>
-    <t>합산 %</t>
-  </si>
-  <si>
-    <t>제안</t>
-  </si>
-  <si>
-    <t>80% 이상</t>
-  </si>
-  <si>
-    <t>강한 매수</t>
-  </si>
-  <si>
-    <t>73% 이상</t>
-  </si>
-  <si>
-    <t>73% 이상 ~ 80% 미만</t>
-  </si>
-  <si>
-    <t>매수</t>
-  </si>
-  <si>
-    <t>67% 이상 ~ 73% 미만</t>
-  </si>
-  <si>
-    <t>약한 매수</t>
-  </si>
-  <si>
-    <t>60% 이상 ~ 67% 미만</t>
-  </si>
-  <si>
-    <t>37% 초과 ~ 67% 미만</t>
-  </si>
-  <si>
-    <t>홀딩</t>
-  </si>
-  <si>
-    <t>33% 초과 ~ 37% 이하</t>
-  </si>
-  <si>
-    <t>약한 매도</t>
-  </si>
-  <si>
-    <t>27% 초과 ~ 33% 이하</t>
-  </si>
-  <si>
-    <t>매도</t>
-  </si>
-  <si>
-    <t>20% 초과 ~ 27% 이하</t>
-  </si>
-  <si>
-    <t>27% 이하</t>
-  </si>
-  <si>
-    <t>강한 매도</t>
-  </si>
-  <si>
-    <t>20% 이하</t>
-  </si>
-  <si>
-    <t>33% 초과 ~ 60% 미만</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>(3개월,6개월,1년 조회에만 적용) 하락 추세선 상승 추세선 모두 하락이면서 해당 시점에 1개월(1시간봉기준)조회시 상승추세선이 상방향일 때</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>(3개월,6개월,1년 조회에만 적용) 하락 추세선 상승 추세선 모두 상승이면서 해당 시점에 1개월(1시간봉기준)조회시 상승추세선이 하방향일 때 상승 추세선에 근접했으면 가점, 하방향 아니면 무효</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>신고가 저항</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>신고가 달성</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>6개월 상승률이 800% 이상이면서 위에 저항이 없는 신고가의 경우</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>6개월 상승률이 800% 미만이면서 위에 저항이 없는 신고가의 경우</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>신고가 이탈</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>신고가 돌파 후 다시 하락 추세선 안으로 현재가가 내려왔을 때</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>점수를 %로 바꾸는 법: 0점이면 0%, 15점(기본)이면 50%, 30점이면 100%.</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>가까운 가격: 하루 변동폭의 약 30%, 또는 주가의 1.0% 중 더 큰 값.</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>한 달동안 15% 이상 25%미만 하락 했을 때</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>한 달 동안 25% 이상 35% 미만 떨어짐</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>한 달 동안 35% 이상 떨어짐</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>점수 규칙 (쉬운 버전) · 지금 앱 v98</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>6개월 동안 800% 이상 오름,횡보 추세나 하락 추세시 무효</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>점수를 %로 바꾸는 법: 1점이면 0%, 15점(기본)이면 50%, 30점이면 100%.</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. 「기본 점수」부터 「신고가 이탈」까지 더합니다.</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>점수 규칙 (쉬운 버전) · 지금 앱 v99</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -854,7 +852,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="26" x14ac:dyDescent="0.65">
       <c r="A1" s="16" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B1" s="17"/>
     </row>
@@ -881,22 +879,22 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
-        <v>3</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.45">
@@ -904,22 +902,22 @@
     </row>
     <row r="12" spans="1:2" ht="20.5" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.45">
@@ -927,17 +925,17 @@
     </row>
     <row r="17" spans="1:1" ht="34" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="34" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="34" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -951,7 +949,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -961,21 +959,21 @@
   <sheetData>
     <row r="1" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>18</v>
       </c>
       <c r="C2" s="5">
         <v>15</v>
@@ -983,10 +981,10 @@
     </row>
     <row r="3" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>21</v>
       </c>
       <c r="C3" s="6">
         <v>-1</v>
@@ -994,10 +992,10 @@
     </row>
     <row r="4" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>22</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>23</v>
       </c>
       <c r="C4" s="5">
         <v>1</v>
@@ -1005,10 +1003,10 @@
     </row>
     <row r="5" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>24</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>25</v>
       </c>
       <c r="C5" s="6">
         <v>-1</v>
@@ -1016,10 +1014,10 @@
     </row>
     <row r="6" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C6" s="5">
         <v>1</v>
@@ -1027,10 +1025,10 @@
     </row>
     <row r="7" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="C7" s="5">
         <v>1</v>
@@ -1038,10 +1036,10 @@
     </row>
     <row r="8" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="C8" s="5">
         <v>1</v>
@@ -1049,10 +1047,10 @@
     </row>
     <row r="9" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>30</v>
       </c>
       <c r="C9" s="5">
         <v>1</v>
@@ -1060,10 +1058,10 @@
     </row>
     <row r="10" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>31</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>32</v>
       </c>
       <c r="C10" s="6">
         <v>-2</v>
@@ -1071,10 +1069,10 @@
     </row>
     <row r="11" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>33</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>34</v>
       </c>
       <c r="C11" s="6">
         <v>-1</v>
@@ -1082,10 +1080,10 @@
     </row>
     <row r="12" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>35</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>36</v>
       </c>
       <c r="C12" s="5">
         <v>1</v>
@@ -1093,10 +1091,10 @@
     </row>
     <row r="13" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>37</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>38</v>
       </c>
       <c r="C13" s="5">
         <v>1</v>
@@ -1104,10 +1102,10 @@
     </row>
     <row r="14" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>39</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>40</v>
       </c>
       <c r="C14" s="6">
         <v>-1</v>
@@ -1115,10 +1113,10 @@
     </row>
     <row r="15" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>41</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>42</v>
       </c>
       <c r="C15" s="5">
         <v>1</v>
@@ -1126,10 +1124,10 @@
     </row>
     <row r="16" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C16" s="6">
         <v>-1</v>
@@ -1137,10 +1135,10 @@
     </row>
     <row r="17" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>44</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>45</v>
       </c>
       <c r="C17" s="5">
         <v>1</v>
@@ -1148,10 +1146,10 @@
     </row>
     <row r="18" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>46</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>47</v>
       </c>
       <c r="C18" s="5">
         <v>1</v>
@@ -1159,10 +1157,10 @@
     </row>
     <row r="19" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>48</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>49</v>
       </c>
       <c r="C19" s="5">
         <v>1</v>
@@ -1170,10 +1168,10 @@
     </row>
     <row r="20" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>50</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>51</v>
       </c>
       <c r="C20" s="6">
         <v>-1</v>
@@ -1181,76 +1179,76 @@
     </row>
     <row r="21" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C21" s="6">
-        <v>-1</v>
+        <v>92</v>
+      </c>
+      <c r="C21" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="C22" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="C23" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="C24" s="5">
-        <v>3</v>
+        <v>100</v>
+      </c>
+      <c r="C24" s="6">
+        <v>-3</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C25" s="6">
-        <v>-3</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>57</v>
+        <v>99</v>
       </c>
       <c r="C26" s="6">
-        <v>-2</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>58</v>
+        <v>98</v>
       </c>
       <c r="C27" s="6">
         <v>-1</v>
@@ -1258,50 +1256,39 @@
     </row>
     <row r="28" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="4" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C28" s="6">
-        <v>-1</v>
+        <v>95</v>
+      </c>
+      <c r="C28" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="4" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="C29" s="5">
-        <v>1</v>
+        <v>96</v>
+      </c>
+      <c r="C29" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="4" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C30" s="6">
         <v>-1</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="C31" s="6">
-        <v>-1</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:C30" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:C29" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1319,21 +1306,21 @@
   <sheetData>
     <row r="1" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="4" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="C2" s="7">
         <v>0</v>
@@ -1341,10 +1328,10 @@
     </row>
     <row r="3" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="4" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C3" s="6">
         <v>-1</v>
@@ -1352,21 +1339,21 @@
     </row>
     <row r="4" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="4" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="4" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="C5" s="7">
         <v>0</v>
@@ -1374,10 +1361,10 @@
     </row>
     <row r="6" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="C6" s="6">
         <v>-1</v>
@@ -1385,10 +1372,10 @@
     </row>
     <row r="7" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>61</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>67</v>
       </c>
       <c r="C7" s="7">
         <v>0</v>
@@ -1396,7 +1383,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" s="18" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
@@ -1425,129 +1412,129 @@
   <sheetData>
     <row r="1" spans="1:5" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A1" s="19" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="B1" s="17"/>
       <c r="D1" s="19" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="E1" s="17"/>
     </row>
     <row r="2" spans="1:5" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="8" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="8" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="9" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="11" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="13" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="13" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="14" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" s="18" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B11" s="17"/>
       <c r="C11" s="17"/>
@@ -1556,7 +1543,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" s="18" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="B12" s="17"/>
       <c r="C12" s="17"/>

</xml_diff>

<commit_message>
Apply sheet v100: period-vs-1m trend, base 12 with 0/12/24 scale, ATH reenter in 5 bars.
</commit_message>
<xml_diff>
--- a/규칙_점수표.xlsx
+++ b/규칙_점수표.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\trade-advisor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D509FC9D-7DD2-4226-87A1-A21F8E72413F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DD66254-6171-46EA-963B-EDDA5D89DE50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <sheet name="매수 매도 기준" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'옵션 점수'!$A$1:$C$7</definedName>
   </definedNames>
   <calcPr calcId="0"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="112">
   <si>
     <t>점수는 아래 항목을 하나씩 보고, 해당되면 더하거나 뺍니다.</t>
   </si>
@@ -38,9 +38,6 @@
     <t>순서</t>
   </si>
   <si>
-    <t>2. 더한 점수를 %로 바꿉니다. 0점이면 0%, 15점(기본)이면 50%, 31점이면 100%.</t>
-  </si>
-  <si>
     <t>3. %로 매수 / 매도 / 홀딩을 정합니다.</t>
   </si>
   <si>
@@ -332,10 +329,6 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>신고가 돌파 후 3봉 이내에 다시 하락 추세선 안으로 현재가가 내려왔을 때, 3봉 이후 무효</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
     <t>1개 봉만에 20% 이상 상승했을 시</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
@@ -348,15 +341,55 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>점수를 %로 바꾸는 법: 1점이면 0%, 15점(기본)이면 50%, 30점이면 100%.</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
     <t>1. 「기본 점수」부터 「신고가 이탈」까지 더합니다.</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>점수 규칙 (쉬운 버전) · 지금 앱 v99</t>
+    <t>조회기간 추세</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>(3개월,6개월,1년 조회에만 적용)조회기간 추세가 상승이면서 1개월 조회시(1시간봉) 상승 추세일때</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>(3개월,6개월,1년 조회에만 적용)조회가간 추세가 상승이면서 1개월 조회시(1시간봉) 하락 추세일때</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>(3개월,6개월,1년 조회에만 적용)조회기간 추세가 하락이면서 1개월 조회시(1시간봉) 상승 추세일 때</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>(3개월,6개월,1년 조회에만 적용)조회기간 추세가 하락이면서 1개월 조회시(1시간봉) 하락 추세일때</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>(3개월,6개월,1년 조회에만 적용)조회기간 추세가 횡보이면서 1개월 조회시(1시간봉) 하락 추세일때</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>(3개월,6개월,1년 조회에만 적용)조회기간 추세가 횡보이면서 1개월 조회시(1시간봉) 상승 추세일 때</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>(3개월,6개월,1년 조회에만 적용)조회기간 추세와 1개월 조회시(1시간봉) 상승 추세일 때</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>점수 규칙 (쉬운 버전) · 지금 앱 v100</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>점수를 %로 바꾸는 법: 0점이하면 0%, 12점(기본)이면 50%, 24점이상이면 100%.</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>2. 더한 점수를 %로 바꿉니다. 0점이하면 0%, 12점(기본)이면 50%, 24점이상이면 100%.</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>신고가 돌파 후 5봉 이내에 다시 하락 추세선 안으로 현재가가 내려왔을 때, 3봉 이후 무효</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -852,7 +885,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="26" x14ac:dyDescent="0.65">
       <c r="A1" s="16" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="B1" s="17"/>
     </row>
@@ -879,22 +912,22 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.45">
@@ -902,22 +935,22 @@
     </row>
     <row r="12" spans="1:2" ht="20.5" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.45">
@@ -925,17 +958,17 @@
     </row>
     <row r="17" spans="1:1" ht="34" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="34" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="34" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -949,7 +982,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -959,43 +992,43 @@
   <sheetData>
     <row r="1" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>17</v>
-      </c>
       <c r="C2" s="5">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="4" t="s">
-        <v>19</v>
+        <v>100</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="6">
+        <v>101</v>
+      </c>
+      <c r="C3" s="5">
         <v>-1</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="4" t="s">
-        <v>21</v>
+        <v>100</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>22</v>
+        <v>102</v>
       </c>
       <c r="C4" s="5">
         <v>1</v>
@@ -1003,21 +1036,21 @@
     </row>
     <row r="5" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="4" t="s">
-        <v>23</v>
+        <v>100</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="6">
+        <v>103</v>
+      </c>
+      <c r="C5" s="5">
         <v>-1</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
-        <v>23</v>
+        <v>100</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="C6" s="5">
         <v>1</v>
@@ -1025,10 +1058,10 @@
     </row>
     <row r="7" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
-        <v>26</v>
+        <v>100</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>86</v>
+        <v>105</v>
       </c>
       <c r="C7" s="5">
         <v>1</v>
@@ -1036,65 +1069,65 @@
     </row>
     <row r="8" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
-        <v>27</v>
+        <v>100</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>87</v>
+        <v>106</v>
       </c>
       <c r="C8" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="4" t="s">
-        <v>28</v>
+        <v>100</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>29</v>
+        <v>107</v>
       </c>
       <c r="C9" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="C10" s="6">
-        <v>-2</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="4" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C11" s="6">
-        <v>-1</v>
+        <v>21</v>
+      </c>
+      <c r="C11" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="4" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C12" s="5">
-        <v>1</v>
+        <v>23</v>
+      </c>
+      <c r="C12" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="4" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="C13" s="5">
         <v>1</v>
@@ -1102,21 +1135,21 @@
     </row>
     <row r="14" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="4" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C14" s="6">
-        <v>-1</v>
+        <v>85</v>
+      </c>
+      <c r="C14" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="4" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>41</v>
+        <v>86</v>
       </c>
       <c r="C15" s="5">
         <v>1</v>
@@ -1124,43 +1157,43 @@
     </row>
     <row r="16" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="4" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C16" s="6">
-        <v>-1</v>
+        <v>28</v>
+      </c>
+      <c r="C16" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="4" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C17" s="5">
-        <v>1</v>
+        <v>30</v>
+      </c>
+      <c r="C17" s="6">
+        <v>-2</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="4" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C18" s="5">
-        <v>1</v>
+        <v>32</v>
+      </c>
+      <c r="C18" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="4" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="C19" s="5">
         <v>1</v>
@@ -1168,87 +1201,87 @@
     </row>
     <row r="20" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="4" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="C20" s="6">
-        <v>-1</v>
+        <v>36</v>
+      </c>
+      <c r="C20" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="4" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="C21" s="5">
-        <v>1</v>
+        <v>38</v>
+      </c>
+      <c r="C21" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="4" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>93</v>
+        <v>40</v>
       </c>
       <c r="C22" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="4" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="C23" s="5">
-        <v>3</v>
+        <v>41</v>
+      </c>
+      <c r="C23" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="4" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="C24" s="6">
-        <v>-3</v>
+        <v>43</v>
+      </c>
+      <c r="C24" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="4" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C25" s="6">
-        <v>-2</v>
+        <v>45</v>
+      </c>
+      <c r="C25" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="4" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="C26" s="6">
-        <v>-1</v>
+        <v>47</v>
+      </c>
+      <c r="C26" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="4" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>98</v>
+        <v>49</v>
       </c>
       <c r="C27" s="6">
         <v>-1</v>
@@ -1256,10 +1289,10 @@
     </row>
     <row r="28" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="4" t="s">
-        <v>89</v>
+        <v>50</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C28" s="5">
         <v>1</v>
@@ -1267,28 +1300,105 @@
     </row>
     <row r="29" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="4" t="s">
-        <v>88</v>
+        <v>50</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="C29" s="6">
-        <v>-1</v>
+        <v>92</v>
+      </c>
+      <c r="C29" s="5">
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="4" t="s">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="B30" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C30" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A31" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C31" s="6">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A32" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C32" s="6">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A33" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B33" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="C30" s="6">
+      <c r="C33" s="6">
         <v>-1</v>
       </c>
     </row>
+    <row r="34" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A34" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C34" s="6">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A35" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C35" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A36" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C36" s="6">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A37" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C37" s="6">
+        <v>-1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C29" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:C36" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1306,21 +1416,21 @@
   <sheetData>
     <row r="1" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="C2" s="7">
         <v>0</v>
@@ -1328,10 +1438,10 @@
     </row>
     <row r="3" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C3" s="6">
         <v>-1</v>
@@ -1339,21 +1449,21 @@
     </row>
     <row r="4" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C5" s="7">
         <v>0</v>
@@ -1361,10 +1471,10 @@
     </row>
     <row r="6" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C6" s="6">
         <v>-1</v>
@@ -1372,10 +1482,10 @@
     </row>
     <row r="7" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C7" s="7">
         <v>0</v>
@@ -1383,7 +1493,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
@@ -1412,129 +1522,129 @@
   <sheetData>
     <row r="1" spans="1:5" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A1" s="19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B1" s="17"/>
       <c r="D1" s="19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E1" s="17"/>
     </row>
     <row r="2" spans="1:5" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>66</v>
-      </c>
       <c r="D2" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>65</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="D3" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="D3" s="8" t="s">
-        <v>69</v>
-      </c>
       <c r="E3" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="D4" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="D4" s="8" t="s">
-        <v>72</v>
-      </c>
       <c r="E4" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="D5" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="D5" s="9" t="s">
-        <v>74</v>
-      </c>
       <c r="E5" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="B6" s="12" t="s">
-        <v>76</v>
-      </c>
       <c r="D6" s="11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="D7" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="D7" s="13" t="s">
-        <v>79</v>
-      </c>
       <c r="E7" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="D8" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="D8" s="13" t="s">
-        <v>81</v>
-      </c>
       <c r="E8" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="B9" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="D9" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="D9" s="14" t="s">
-        <v>84</v>
-      </c>
       <c r="E9" s="15" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" s="18" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="B11" s="17"/>
       <c r="C11" s="17"/>
@@ -1543,7 +1653,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" s="18" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B12" s="17"/>
       <c r="C12" s="17"/>

</xml_diff>